<commit_message>
Stable pipeline with duration validation (Clean push)
</commit_message>
<xml_diff>
--- a/Curriculum Plus Product Videos.xlsx - Sheet1.xlsx
+++ b/Curriculum Plus Product Videos.xlsx - Sheet1.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>Fixed &amp; Compressed</t>
+          <t>Fixed without compression</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -571,12 +571,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>02:20-02:32, 03:22-03:59</t>
+          <t>03:22-03:39</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>hry | are | U  wuQ:,=© r ) Crucis Content r ) Erdocrine  ENTIRE 2QAC TI!  Tue, November 22, 2022  TEST It ya OREREQLISIE te the segue | U  wuQ:,=© e@ Crucis Content r ) Erdocrine  ENTIRE 2QAC TI!  Tue, November 22, 2022  TES) It ya OREREQLISTE te the sesuine | U  e@ Crucis Content e@ Erdocrine  ENTIRE PRACTICA TEST In ya ORE  Tue, November 22, 2022  REOLIM  je the seyuige | U  Crucis Content  Eedocnne  ENTIRE PRACTICA TEST In ya ORE  Tue, November 22, 2022  REOLIM  je the seyuige | Help | U  e@ Crucis Content r ) Erdocrine  ENTIRE PRACTICA TEST In ya ORE  Tue, November 22, 2022  REOLIM  je the sexo | U  ww, e@ Cues Content r ) Erdoctine  ENTIRE 22AC TIE  Tue, November 22, 2022  TEST Iya OREREQLISITE te the segue | ENTIRE 22 AC TILE TEST It ya PREREOLISE  je the sexo  Tue, November 22, 2022 | U  wuQ:,=© e@ Crucis Content r ) Erdocrine  ENTIRE 2QAC TI!  Tue, November 22, 2022  TEST It ya OREREQLISIE te the segue | U  ww, e@ Crucis Content r ) Erdocrine  ENTIRE 22AC TIE!  Tue, November 22, 2022  TEST It ya PREREQUISITE te the sesuoe | U  wo“ e@ Crucis Content r ) Erdocrine  ENTIRE 2QAC TI!  Tue, November 22, 2022  TES) It ya OREREQLISTE te the sesuine | U  wC““lHD= e@ Crucis Content r ) Erdocrine  ENTIRE 2QAC TI!  Tue, November 22, 2022  TEST It ya OREREQLISIE te the segue | U  w30wre e@ Crucis Content r ) Erdocrine  ENTIRE 22AC TI!  Tue, November 22, 2022  TES) It ya OREREQLISTE te the segue | U  e@ Crucis Content r ) Erdocrine  ENTIRE PRAC TICS TEST I ya ORE  Tue, November 22, 2022  REOLIM  je the sexo | U  e@ Crucis Content r ) Erdocrine  ENTIRE PRACTICE TEST In ya ORE  Tue, November 22, 2022  REOLIM  je the sexo</t>
+          <t>Ith | ard | create | your | Gwn | NCLEX | pan | AKE | ENTIRE | TEST | the | Tue, | November | 2022 | Content | ord | yout | Cwn | study | Its | you | thas | PRACTICE | TIC! | Own | own | Help</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>Fixed &amp; Compressed</t>
+          <t>Fixed without compression</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -628,12 +628,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>00:49-00:51, 01:19-02:45, 03:12-03:35, 03:56-04:13, 05:21-05:53, 06:11-06:12</t>
+          <t>00:49-02:45, 03:12-03:35, 03:55-04:03, 05:21-05:53</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Help | Phare Borers | se eta MedKat ons (42) P) 20 ‘Study Now  zal Med cations (27; f a 20 Study Now | ‘active Channel sessions covering content and strategy | NCLEX - Acute Post-Traumatic Stress Disorder  NCLEX - Urinary System Tests | Nursing School - Abscess. | Video 5m + Stress Reduction  Video ?5m  2 Dranarnn ies tho Evam | &gt; + Live, interactive Channel JN Covering Content and strategy | Video 5m + Stress Reduction  video 25m  Dranannn tee tha Evam | Nursing School - Abdominal Surgery  Nursing School - Abdominal Trauma | Nursing School - Abscess  Nursing School - Absorption | Nursing Schoot - Abnormal Involuntary Movement Scale (AIMS)  Nursing School - Abscess  Nureing Schnol . Ahcorotion | Video rr + Stress Reduction  Video ?5m | TAKE ME THERE MARK COMPLETE | se eta Medxations (42) fe) 20 ‘Study Now  zal Med cations (27; Ce) 20 Study Now | NCLEX - Urolithiasis um  NCLEX - Violent/Aggressive Behavior an  Biricy thesen:me | Cardio 1.1 - ECG Interpretation Review  Tass cab chaste bey ae  etatierapee nag tl tir heat ang tak pace ot the | Cardio 1.1 - ECG Interpretation Review  rab Heatatee EO at  C15 te tar heat tol vy tak pace tthe | Nursing School - Abscess | WATCH | 7 [ en tent  Normal Labor and Delivery e Karma Lityquist 12:30 PM - 12:20 AM IST e Fazoce ne In tas sewer a tune educatit an ‘enw a cane study and d cuss facto “4  alnoatae  effestirg 1¢ lbor prccess We el abo dn os assets mes and nats 15 SS BB bree ee fe NOE. imterveanens ‘or a cert cuerg Lor aed te wety | “here ave toral B97 cardsin your cecks | Video 5m + Stress Reduction  Video 25m  Dranannn tee tha Evam | NCLEX - Water-Soluble Vitamins  NCLEX - Women’s Health Medications | MARK COMPLETE | WATC!  Benen Pate | ee. Normal Labor and Delivery 8 Kara. lyquat 11 WORM 12 204M Ss”  eS keen ee ee ec er ce  eg tae lugar pene | “here ae toral B97 cardsin your cecks | Phare Forces | Video 5m + Stress Reduction  video 25m  Dranarnn ine tha Evam | Normal Labor and Delivery one 110M 12 204M S°  [con ee eer ney  sMecbeg tae liter pe iey aE I aes | atric (ol)  Juctive (71) | Juctive (71) | Quiz 36rr I mec + Kaplan Cardiovascular B NGN  Que 36 Tmee + Kaplan Cardiovascular C NGN | Quiz 36m Tmec + Kaplan Cardiovascular B NGN  Que 36m Tmee + Kaplan Cardiovascular C NGN | atric (or)  Juctive (71) | Quiz 36 Tmec + Kaplan Cardiovascular B NGN  Quiz 36m Tmec + Kaplan Cardiovascular C NGN | Quiz 36rr Timed + Kaplan Cardiovascular B NGN  Quiz 36 Tmee + Kaplan Cardiovascular C NGN | Quiz 36 Timed + Kaplan Cardiovascular B NGN  Quiz 36 Tmee + Kaplan Cardiovascular C NGN | Quiz 36 Timed + Kaplan Cardiovascular B NGN  Que 36 Tmee + Kaplan Cardiovascular C NGN | Quiz 36m = Timed + Kaplan Cardiovascular B NGN  Quiz 36m = Timea + Kaplan Cardiovascular C NGN | Quiz 36m Timed + Kaplan Cardiovascular B NGN  Quiz 36m Timed + Kaplan Cardiovascular C NGN | pus syruree  agas | Question 3 Severa ours a‘ter be rg advirted to the ut ar  Phys 0 of cas Integr  Pharna Therapies  ag Ca Pareste-al  Medicat ons Sod. Tracnel Merkers | Question 3 Severa nours a’ter be rg admitted to the wrt, ar  Phys 00g cal Integr y  Pharnace og ca /Pa-enteral Therapies  Medizators $od 2 Tracrnel Blockers | OT OTTTT TG Qos, WET TEs UP  Question 2 When the aurse performs CPR cr an ad IPowack cthe -erre-t ranc  Phrys 0 og cul Integt  Phys 0 og cel Adupistion  Lara epi rotary Resse tat 99 678} | Question 2 Wren the 1urse performs CPR cr anadult, wich s the correct ratic  Phys 0 0g cal Integr sy  Phys 0 0g cal Adaptation  Cera ope moray Resse tat a7 FPR) | Nvesuen s Severa ours a‘ter he rg advirted to tne ut ar  QKuecian 4  Phys 0 og cel Integr 5y  Pharnass Therapies  3g Ca Parente-al | Question 2  Ween the vurse performs CPRcr  Fhys og cal integrsy Phys 0 og cal Adaptatior ee cee money aoc aradult, wich s the correct ratic SSESEL TURES) | bus syrorcne  agas | BREN EME BE  “  Be NN an adult. wich -s the correct ratic  Question 3 Severa hours after berg  PINS? O Os Gal TIER! -y  Er ancrcal Intaor  Pharnacalyg ca Pare~reral  Resse tat on  Medizat ons Sod  Bevirw | 3/Overview | « Elderty; Pregnancy &amp; Lactation  « Liver &amp; Renal Disease _ &amp; adhe mens facdian Banama'| base  pyencs  Waions and Contraindications: | im level osety essure closely n elderly chants hn extended-reiease tablets, | asias ventnoular contractions.  feonllator: | pus syndrome.  asias. ventneular contractions. | el * Flecainide (Tambocor) | e@ Deransafannnas (Bhuthmanii | « Astnma; Cardiac Pacemaker + Medication Interactions | pus syndrome.  asias. ventricular contractions. | * FPropatenone (Rhytnmol J + Supraventricular Dysrhythmias a Dysrhythmlas | a/Overviow | amas ventnoular contractions.  finllavon, | im level closely essure closely in elderty chents. | finllaton, | + Supraventricular Dysrhythmias  lar Dysrhythmias | Elderty; Pregnancy &amp; Lactation Liver &amp; Renal Disease  Asthma; Cardiac Pacemaker Marit-atinn intararctinne | ¢ Flecainide (Tambocor) * Propafenone (Rhythmol)  * Supraventricular Dysrhythmias ] | * Medication interactions ]  KAPLAN) NURSING | + Flecainide (Tambocor) + Propafenone (Rhythmol) | elidel Se ed  extended ‘eloase tat ets | ions and Contraindications:  « Elderty; Pregnancy &amp; &amp; Lactation | im level closely essure close'y in elderly chants h extendedtolease taricts | + Liver &amp; Rena! Disease « Asthma; Cardiac Pacemaker + Medication Interactions | KAPLAN) NURSING | bus syndrome  asias  yventncular contractions. | wer!</t>
+          <t>THERE | aed | strategy | MARK | Absorption | Media | Acute | and | interactive | Scale | Delivery | (AIMS) | ‘Study | Urolithiasis | Abdominal | Labor | IST | tee | Urinary | Water-Soluble | study | Involuntary | Abscess | Help | tir | 12:20 | Review | 12:30 | NCLEX | Interpretation | Study | dnc | Reduction | Normal | Cardio | cuerg | Health | aho | Channel | Surgery | ine | Vitamins | Now | your | aal | the | Abnormal | covering | content | Karma | Nursing | Card | WATCH | Med | Tests | School | Behavior | Violent/Aggressive | 204M | ons | cations | Evam | tho | Medications | COMPLETE | link | Video | OSE | iske | B97 | Disorder | Otitis | Stress | TAKE | ECG | Movement | Live, | gical | Post-Traumatic | tha | sessions | Schoot | System | tar | video | oductive | Cardiovascular | Quiz | NGN | 36m | Timea | performing | CPR, | which | the | When | nurse | performs | CPRON | Physi | serform | Question | CPR | cul | Phys | cel | tat | Wren | wich | correct | ratic | cal | Cal | Ween | Adaptatior | Severa | hours | berg | Adaptation | Resusc | Sod | Integr | wes | nours | ours | tne | Therapies | cose | lupus | dosely | Pacemaker | Medication | Disease | syndrome. | jum | ush | Supraventricular | ventncular | Asthma; | syndrome | and | contractions. | Propafenone | Dysrhythmlias | ventricular | der | Dysrhythmias | closety | chents. | (Rhythmol) | Renal | Liver | NURSING | Interactions | Pressure | Flecainide | (Tambocor) | ium | Lactation | elderty | level | closely | ions | elderly | Pregnancy | Cardiac | Elderty; | contractions | lar | Contraindications: | pressure | chents</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>Fixed &amp; Compressed</t>
+          <t>Fixed without compression</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -685,12 +685,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>00:29-00:30, 01:47-03:33, 04:42-04:57, 05:38-05:39</t>
+          <t>01:47-03:33</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>ye ’ “ag | eee ene NE  &gt;rep Class  telp | en eee  *rep Class  delp | ee ee Ee  *rep Class  delp | een Oe eee  rep Class  delp | eee  ?rep Class  telp | eee  &gt;rep Class  telp | ee Oe eee  &gt;rep Class  delp | eerie a ciel initial  &gt;rep Class  telp | eee eedeleciearietel inieieiei  &gt;rep Class  telp | ee een eee ee ee eee  rep Class  delp | ee een ee  &gt;rep Class  delp | eee NN  &gt;rep Class  telp | eerie a ciel initial  rep Class  telp | nen  &gt;rep Class  telp | ee NN TO  &gt;rep Class  telp | Question Trainers 1-3  Diagnostic Test | Roadmap To Success  ?hase Three: After Kaplan | Roadmap To Success  ?hase Three: After Kaplan  ad | Roadmap To Success  ?hase Three: After Kaplan  - of | 3oadmap To Success  ?hase Three: After Kaplan | Roadmap To Success  ?hase Three: After Kaplan  —™ | %eadiness Test  VGN Challenge Tests | eadiness Test  VGN Challenge Tests | eadiness Test  IGN Challenge Tests | 3eadiness Test  VGN Challenge Tests | mu)  my cit mh Ha a | he an  ra tt uhh | vl te a | pa! oo D ei io a ar</t>
+          <t>Phase | Three: | After | Prep | Class | Help | Question | Trainers | Diagnostic | Test | Roadmap | Success | Readiness | Tes? | NGN | Challenge | Tests</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Fixed &amp; Compressed</t>
+          <t>Fixed without compression</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Turther teaching neeaed¢ | Turther teaching neeaed + | Turther teacning neeaed?+ | Turther teaching neeaed? | Turther teacning neeaed¢ | Turther teacning neeaed + | Turther teacning neeaed?</t>
+          <t>further | teaching | needed?</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Fixed &amp; Compressed</t>
+          <t>Fixed without compression</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>ne THC CUT QUT Or PN TTT Infection Control Risk Potential | ne THC CUT QUT Or PN EIT Infection Control Risk Potential | ns THOU TT QUT Ot PN ITT Infection Control Risk Potential | BO THC CUT QUT Ot PN TTT VT Infection Control Risk Potential | BO TH CCUGTT QUT Or DN TTT MT Infection Control Risk Potential | ne TH CCUG TT QUT Ot PN TTT MT Infection Control Risk Potential | BO TH CCUG TT QUT Ot PN TTT MT Infection Control Risk Potential | ns THC CUT QUT Ot DTT MT Infection Control Risk Potential | ne TCU TT QUT Or PTT MT Infection Control Risk Potential | BO TCU TT QUT Ot PTT MT Infection Control Risk Potential | Bn THC CUT QUT Or PITT MT Infection Control Risk Potential | ns WHC CUT QUT Or PN ITT MT Infection Control Risk Potential | ne TCU TT QUT Ot PIT Infection Control Risk Potential | Bn TWHCCUG TT QUT Or PNRM MT Infection Control Risk Potential | ne THCCUG TT QUT Or PN INSTT MT Infection Control Risk Potential | BO TCU TT QUT Or PIT MT Infection Control Risk Potential | CB TWHCCUGTT QUT Ot PITT ST Infection Control Risk Potential | ne TWHCCUGTT QUT OT PR INSTT MT Infection Control Risk Potential | ns THECUTUP OT PITT MT Infection Control! Risk Potential | ns TH CCUGTT QUT OT PTT Infection Control Risk Potential | ne THCCUG TT QUT OT PN INSTT MT Infection Control Risk Potential | ne TH CCUGTT QUT Or PR ITT MT Infection Control Risk Potential | ne THC CUT QUT Ot PN TTT MT Infection Control Risk Potential | ne TH CCUGT QUT Ot PITT MT Infection Control Risk Potential | rs THC CUT QUT Or PN TTT Infection Control Risk Potential | ne TH CCUGTT QUOT PERT VT Infection Control Risk Potential | ns THC CUG TT QUT Or PN ITT Infection Control Risk Potential | ne THC CUT QUT Or PN ITT Infection Control Risk Potential | ne THC CUT QUT Or TN ITT ST Infection Control Risk Potential | ne THC CUT QUT Or PNET Infection Control Risk Potential | ne TCU TT QUT Or PNR ITT Infection Control Risk Potential | ne THC CUT QUT Ot PN ITT Infection Control Risk Potential | BO THOU TT QUT Or PN TT Infection Control Risk Potential | ne THC CUT QUT Ot PITT Infection Control Risk Potential | ns THOU TT QUT Or PITT Infection Control Risk Potential | ne THOU TT QUT Or PN ITT Infection Control Risk Potential | ns THC UU TT QUT Ot PITT Infection Control Risk Potential | BO THC CUG TT QUT Ot PN TTT Infection Control Risk Potential | ne THOU TT QUT Or PNET Infection Control Risk Potential | BO THECUTUP Or PNET Infection Control Risk Potential | ns THOU TT QUT Or PNR ITT Infection Control Risk Potential | ne THCCUGTT QUT OT PTT Infection Control Risk Potential | ne THC CUT QUT Or PTT Infection Control Risk Potential | ne THC CUT QV Or PS TTT Infection Control Risk Potential | ns THC CUT QUT Or PTT Infection Control Risk Potential | ne THC CUGTT QUT Ot PS TTT Infection Control Risk Potential | ns THC CUT QUT Or PN ITT Infection Control Risk Potential | ns THC CUGTT QUT Or PN TT Infection Control Risk Potential | Bn THC CUT QUT Or PN ITT Infection Control Risk Potential | ns TCU TT QUT Ot PN ITT Infection Control Risk Potential | BO THC CUT QUT Or PN EIT Infection Control Risk Potential | ne THC CUT QUT Or PNR ITT Infection Control Risk Potential | ns TCU TT QUT Or PNET Infection Control Risk Potential | ne THC CUT QUT Or PNT Infection Control Risk Potential | ns THC CUT QUT Or PNT Infection Control Risk Potential | ne TCU TT QUT Ot PNT MT Infection Control Risk Potential | ns TCU QUT Or PITT Infection Control Risk Potential | ne THCCUG TT QUOTE OT PITT MT Infection Control Risk Potential | ns THCCUG TT QUT Or PITT MT Infection Control Risk Potential | ne THCCUG TT QUT Or PN TTT MT Infection Control Risk Potential | ne THCCUG TT QUT OT PITT MT Infection Control Risk Potential | BO THC CUGTT QUT Ot PN TT Infection Contro! Risk Potential | Bn THC CUT QUT Ot PN Infection Contro! Risk Potential | ne THECUTUP Or PN TTT Infection Control Risk Potential | ns THC CUT QUT Ot PTT Infection Control Risk Potential | ns TH CCUG TT QUT Or PNET Infection Control Risk Potential | ns THC CUT QUT Or PN TT Infection Control Risk Potential | ne TCU TT QUT Or PN I Infection Control Risk Potential | ne THC CUT QUT Ot PN Infection Control Risk Potential | ns THC CUT QUT Or PNET Infection Control Risk Potential | ne THC CUT QUT Ot PN TT Infection Control Risk Potential | rs THC CUGTT QUT Or TN TTT MT Infection Control Risk Potential | rn THOU QUT Ot PN TTT Infection Control Risk Potential | BT TCU TT QUT Or TN ETT Infection Control Risk Potential | BT THOU TT QUT Or PN ITT Infection Control Risk Potential | CB THC CUGTT QUT Or PNET Infection Control Risk Potential | ne TWHCCUGTT QUT OT DTT MT Infection Control Risk Potential | ne THC CUT QUT Or PITT MT Infection Control Risk Potential | ne WHC CUT QUT Ot PN ITT MT Infection Control Risk Potential | ne WHC CUT QUT Or PTT MT Infection Control Risk Potential | BO THC CUT QUT Or PITT MT Infection Control Risk Potential | ne TCU TT QUT Ot PTT MT Infection Control Risk Potential | ne THC CUT QUT Or PTT MT Infection Control Risk Potential | ne TCU TT QUT Ot PN ETT MT Infection Control Risk Potential | BO TCU TT QUT Ot PN TT MT Infection Control Risk Potential | BO WHC CUT QUT Or PTT Infection Control Risk Potential | BO WHC CUT QUT Or PN TTT MT Infection Control Risk Potential | BO THC CUT QUT Or PITT Infection Control Risk Potential | ne THC CUT QUT Ot PN ITT MT Infection Control Risk Potential | BO TCU TT QUT Or PS TTT MT Infection Control Risk Potential | ne TH CCUGTT QUT Or PN TTT MT Infection Control Risk Potential | BO TCU TT QUT Ot DN TTT MT Infection Control Risk Potential | ns TH CCUG TT QUT Ot DN TTT MT Infection Control Risk Potential | ne TH CCUG TT QUT Ot DN TTT MT Infection Control Risk Potential | ns TH CCUGTT QUT Or PN ITT MT Infection Control Risk Potential | ns TH CCUGTT QUT Ot PN ITT MT Infection Control Risk Potential | BO TH CCUGTT QUT Ot PN TTT MT Infection Control Risk Potential | ns TH CCUGTT QUT Ot PNR TT MT Infection Control Risk Potential | ne TCU TT QUT Ot PN ITT MT Infection Control Risk Potential | Number of items</t>
+          <t>Safety | and | Infection | Control | neauction | Risk | Potential | necuction | ReGUCTION | Number | items</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">

</xml_diff>